<commit_message>
Added new RDF data schemes and visual schemes for economy-table90-94, and fixed XLSX spreadsheet for economy-table91
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table91.xlsx
+++ b/sources/table_normalization/xlsx/economy-table91.xlsx
@@ -98,7 +98,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,8 +164,15 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,6 +191,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -337,6 +350,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -352,51 +396,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -713,64 +726,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
       <c r="F3" s="8"/>
       <c r="G3" s="7"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
     <row r="5" spans="1:9" ht="29">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="30"/>
+      <c r="C5" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="33" t="s">
+      <c r="E5" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="16">
+      <c r="A6" s="27">
         <v>2012</v>
       </c>
-      <c r="B6" s="17"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="3">
         <v>28788</v>
       </c>
@@ -783,10 +796,10 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="16">
+      <c r="A7" s="27">
         <v>2013</v>
       </c>
-      <c r="B7" s="17"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="3">
         <v>71083</v>
       </c>
@@ -799,10 +812,10 @@
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="16">
+      <c r="A8" s="27">
         <v>2014</v>
       </c>
-      <c r="B8" s="17"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="3">
         <v>147172</v>
       </c>
@@ -881,7 +894,7 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="13">
+      <c r="A13" s="24">
         <v>2016</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -899,7 +912,7 @@
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="14"/>
+      <c r="A14" s="25"/>
       <c r="B14" s="4" t="s">
         <v>7</v>
       </c>
@@ -915,7 +928,7 @@
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="14"/>
+      <c r="A15" s="25"/>
       <c r="B15" s="4" t="s">
         <v>8</v>
       </c>
@@ -931,7 +944,7 @@
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="15"/>
+      <c r="A16" s="26"/>
       <c r="B16" s="4" t="s">
         <v>9</v>
       </c>
@@ -947,7 +960,7 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="13">
+      <c r="A17" s="24">
         <v>2017</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -965,7 +978,7 @@
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="14"/>
+      <c r="A18" s="25"/>
       <c r="B18" s="4" t="s">
         <v>7</v>
       </c>
@@ -981,7 +994,7 @@
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="14"/>
+      <c r="A19" s="25"/>
       <c r="B19" s="4" t="s">
         <v>8</v>
       </c>
@@ -997,7 +1010,7 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="15"/>
+      <c r="A20" s="26"/>
       <c r="B20" s="4" t="s">
         <v>9</v>
       </c>
@@ -1031,19 +1044,19 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30">
+      <c r="B22" s="32"/>
+      <c r="C22" s="33">
         <f>SUM(C6:C21)</f>
         <v>1530697</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="33">
         <f>SUM(D6:D21)</f>
         <v>776880</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="33">
         <f>E21</f>
         <v>874379</v>
       </c>
@@ -1053,48 +1066,48 @@
       <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="13" t="s">
         <v>5</v>
       </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
     </row>
     <row r="26" spans="1:7" ht="44.25" customHeight="1">
-      <c r="A26" s="26" t="s">
+      <c r="A26" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
     </row>
     <row r="27" spans="1:7" ht="60" customHeight="1">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
     </row>
     <row r="29" spans="1:7">
       <c r="C29" s="2"/>
@@ -1104,16 +1117,16 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A17:A20"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A17:A20"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>

</xml_diff>